<commit_message>
fun stuff all around
</commit_message>
<xml_diff>
--- a/outputs/enemy-catalogue-20261019/Ashen-Meadows-Enemy-Catalogue.xlsx
+++ b/outputs/enemy-catalogue-20261019/Ashen-Meadows-Enemy-Catalogue.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1" sheetId="1" r:id="R55ec6890e56548b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 2" sheetId="2" r:id="R8a2d4ca78e3b46fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 3" sheetId="3" r:id="R17d39f2a3d834b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 4" sheetId="4" r:id="R59c33e63b23e429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 5" sheetId="5" r:id="R6542cde9567a4005"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boss scaling" sheetId="6" r:id="R2abc8c6be9604921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wildlife and notes" sheetId="7" r:id="R8f78de8da4d64471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1" sheetId="1" r:id="R6833e11093df4af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 2" sheetId="2" r:id="R56880f51c3744922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 3" sheetId="3" r:id="R6256e178452a4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 4" sheetId="4" r:id="Raf17156d329e46eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 5" sheetId="5" r:id="R5c1b2c9aa6a64f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boss scaling" sheetId="6" r:id="Ra1a1f6493c644900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wildlife and notes" sheetId="7" r:id="R84913cc2872c4664"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -568,7 +568,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>1 entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
+        <x:v>1 tier entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -2401,7 +2401,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R453b1e40db39404a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab4b73e1b92942d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2473,7 +2473,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>24 entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
+        <x:v>24 tier entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -4858,7 +4858,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9be89b398dec40a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7aa25b79c35d422b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4930,7 +4930,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>18 entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
+        <x:v>18 tier entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -5635,7 +5635,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="F24" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="G24" s="17" t="str">
         <x:v>Refusal / aggression</x:v>
@@ -7171,7 +7171,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0c99d206942485c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e08349db8e4fbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7243,7 +7243,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>22 entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
+        <x:v>22 tier entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -9580,7 +9580,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a1112a14b0c450a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb0449a4df0d4798"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9652,7 +9652,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>22 entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
+        <x:v>22 tier entries. Current game, 19 October 2026. Damage is before player armor/talents; speed is normal chase unless noted.</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -10506,7 +10506,7 @@
         <x:v>5000</x:v>
       </x:c>
       <x:c r="E28" s="15" t="str">
-        <x:v>Adds; 20% incoming during wave</x:v>
+        <x:v>Summoned adds</x:v>
       </x:c>
       <x:c r="F28" s="16" t="n">
         <x:v>0.5</x:v>
@@ -10518,7 +10518,7 @@
         <x:v>Repeatable pumping-chamber mega hunt</x:v>
       </x:c>
       <x:c r="I28" s="17" t="str">
-        <x:v>Three 210-HP nests; waves of 3 + 2 per surviving nest.</x:v>
+        <x:v>Three 210-HP nests; waves of 3 + 2 per surviving nest; takes 20% damage during waves.</x:v>
       </x:c>
       <x:c r="J28" s="17" t="str">
         <x:v>Break nests and clear the wave for a 12s vulnerability window.</x:v>
@@ -11989,7 +11989,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c48ec7a754e498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ab214d0d9a8489a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12409,7 +12409,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdea3ab7959b24505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dc4dfb092c247a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13074,7 +13074,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d7c9043d2484b85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45579f3c21834f8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>